<commit_message>
update data financial market 2026-02-10
</commit_message>
<xml_diff>
--- a/000_data/008_current_index_basket_msci_colcap_index_col.xlsx
+++ b/000_data/008_current_index_basket_msci_colcap_index_col.xlsx
@@ -366,13 +366,13 @@
         </is>
       </c>
       <c s="5" r="D7">
-        <v>0.0004288974398747</v>
+        <v>0.0004274816696200</v>
       </c>
       <c s="6" r="E7">
-        <v>33040</v>
+        <v>41300</v>
       </c>
       <c s="7" r="F7">
-        <v>0.0077677005204471</v>
+        <v>0.0073684971912924</v>
       </c>
       <c s="1" t="str" r="G7"/>
       <c s="1" t="str" r="H7"/>
@@ -390,13 +390,13 @@
         </is>
       </c>
       <c s="5" r="D8">
-        <v>0.0081611750080083</v>
+        <v>0.0080809857744963</v>
       </c>
       <c s="6" r="E8">
-        <v>4920</v>
+        <v>4960</v>
       </c>
       <c s="7" r="F8">
-        <v>0.0220098343708345</v>
+        <v>0.0167285150902967</v>
       </c>
       <c s="1" t="str" r="G8"/>
       <c s="1" t="str" r="H8"/>
@@ -414,13 +414,13 @@
         </is>
       </c>
       <c s="5" r="D9">
-        <v>0.0112268533819226</v>
+        <v>0.0110877031049725</v>
       </c>
       <c s="6" r="E9">
-        <v>10920</v>
+        <v>13660</v>
       </c>
       <c s="7" r="F9">
-        <v>0.0672016087805842</v>
+        <v>0.0632126011218339</v>
       </c>
       <c s="1" t="str" r="G9"/>
       <c s="1" t="str" r="H9"/>
@@ -438,13 +438,13 @@
         </is>
       </c>
       <c s="5" r="D10">
-        <v>0.0043955028441629</v>
+        <v>0.0043809934962335</v>
       </c>
       <c s="6" r="E10">
-        <v>57000</v>
+        <v>82100</v>
       </c>
       <c s="7" r="F10">
-        <v>0.137335369955539</v>
+        <v>0.150116053789747</v>
       </c>
       <c s="1" t="str" r="G10"/>
       <c s="1" t="str" r="H10"/>
@@ -453,22 +453,22 @@
       <c s="1" t="str" r="A11"/>
       <c s="4" t="inlineStr" r="B11">
         <is>
-          <t xml:space="preserve">CNEC</t>
+          <t xml:space="preserve">CORFICOLCF</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C11">
         <is>
-          <t xml:space="preserve">CANACOL ENERGY LTD</t>
+          <t xml:space="preserve">CORPORACION FINANCIERA COLOMBIANA S.A.</t>
         </is>
       </c>
       <c s="5" r="D11">
-        <v>0.0003530857000916</v>
+        <v>0.0014886982514530</v>
       </c>
       <c s="6" r="E11">
-        <v>5320</v>
+        <v>19740</v>
       </c>
       <c s="7" r="F11">
-        <v>0.0010296526511179</v>
+        <v>0.0122649335702617</v>
       </c>
       <c s="1" t="str" r="G11"/>
       <c s="1" t="str" r="H11"/>
@@ -477,22 +477,22 @@
       <c s="1" t="str" r="A12"/>
       <c s="4" t="inlineStr" r="B12">
         <is>
-          <t xml:space="preserve">CORFICOLCF</t>
+          <t xml:space="preserve">ECOPETROL</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C12">
         <is>
-          <t xml:space="preserve">CORPORACION FINANCIERA COLOMBIANA S.A.</t>
+          <t xml:space="preserve">ECOPETROL S.A.</t>
         </is>
       </c>
       <c s="5" r="D12">
-        <v>0.0014936286492979</v>
+        <v>0.0848171169000947</v>
       </c>
       <c s="6" r="E12">
-        <v>17300</v>
+        <v>2250</v>
       </c>
       <c s="7" r="F12">
-        <v>0.0141640587357777</v>
+        <v>0.079648462663016</v>
       </c>
       <c s="1" t="str" r="G12"/>
       <c s="1" t="str" r="H12"/>
@@ -501,22 +501,22 @@
       <c s="1" t="str" r="A13"/>
       <c s="4" t="inlineStr" r="B13">
         <is>
-          <t xml:space="preserve">ECOPETROL</t>
+          <t xml:space="preserve">EXITO</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C13">
         <is>
-          <t xml:space="preserve">ECOPETROL S.A.</t>
+          <t xml:space="preserve">ALMACENES EXITO S.A.</t>
         </is>
       </c>
       <c s="5" r="D13">
-        <v>0.0850980214621611</v>
+        <v>0.0024541779861055</v>
       </c>
       <c s="6" r="E13">
-        <v>1725</v>
+        <v>4870</v>
       </c>
       <c s="7" r="F13">
-        <v>0.0804650976924158</v>
+        <v>0.0049882290943419</v>
       </c>
       <c s="1" t="str" r="G13"/>
       <c s="1" t="str" r="H13"/>
@@ -525,22 +525,22 @@
       <c s="1" t="str" r="A14"/>
       <c s="4" t="inlineStr" r="B14">
         <is>
-          <t xml:space="preserve">ETB</t>
+          <t xml:space="preserve">GEB</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C14">
         <is>
-          <t xml:space="preserve">EMPRESA DE TELECOMUNICACIONES DE BOGOTA S.A. E.S.P.</t>
+          <t xml:space="preserve">GRUPO ENERGIA BOGOTA S.A. E.S.P.</t>
         </is>
       </c>
       <c s="5" r="D14">
-        <v>0.0036742383201635</v>
+        <v>0.0473482225530609</v>
       </c>
       <c s="6" r="E14">
-        <v>52.5</v>
+        <v>2910</v>
       </c>
       <c s="7" r="F14">
-        <v>0.0001057366645153</v>
+        <v>0.0575053224441498</v>
       </c>
       <c s="1" t="str" r="G14"/>
       <c s="1" t="str" r="H14"/>
@@ -549,22 +549,22 @@
       <c s="1" t="str" r="A15"/>
       <c s="4" t="inlineStr" r="B15">
         <is>
-          <t xml:space="preserve">GEB</t>
+          <t xml:space="preserve">GRUBOLIVAR</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C15">
         <is>
-          <t xml:space="preserve">GRUPO ENERGIA BOGOTA S.A. E.S.P.</t>
+          <t xml:space="preserve">GRUPO BOLIVAR S.A.</t>
         </is>
       </c>
       <c s="5" r="D15">
-        <v>0.0475050344349899</v>
+        <v>0.0002807823840129</v>
       </c>
       <c s="6" r="E15">
-        <v>2975</v>
+        <v>92000</v>
       </c>
       <c s="7" r="F15">
-        <v>0.0774685786726533</v>
+        <v>0.0107812485462055</v>
       </c>
       <c s="1" t="str" r="G15"/>
       <c s="1" t="str" r="H15"/>
@@ -573,22 +573,22 @@
       <c s="1" t="str" r="A16"/>
       <c s="4" t="inlineStr" r="B16">
         <is>
-          <t xml:space="preserve">GRUBOLIVAR</t>
+          <t xml:space="preserve">GRUPOARGOS</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C16">
         <is>
-          <t xml:space="preserve">GRUPO BOLIVAR S.A.</t>
+          <t xml:space="preserve">GRUPO ARGOS S.A.</t>
         </is>
       </c>
       <c s="5" r="D16">
-        <v>0.0002816704163740</v>
+        <v>0.0055421919263986</v>
       </c>
       <c s="6" r="E16">
-        <v>74040</v>
+        <v>18100</v>
       </c>
       <c s="7" r="F16">
-        <v>0.0114315896489302</v>
+        <v>0.0418669679457996</v>
       </c>
       <c s="1" t="str" r="G16"/>
       <c s="1" t="str" r="H16"/>
@@ -597,22 +597,22 @@
       <c s="1" t="str" r="A17"/>
       <c s="4" t="inlineStr" r="B17">
         <is>
-          <t xml:space="preserve">GRUPOARGOS</t>
+          <t xml:space="preserve">GRUPOSURA</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C17">
         <is>
-          <t xml:space="preserve">GRUPO ARGOS S.A.</t>
+          <t xml:space="preserve">GRUPO INVERSIONES SURAMERICANA</t>
         </is>
       </c>
       <c s="5" r="D17">
-        <v>0.0055986348642978</v>
+        <v>0.0021380554898841</v>
       </c>
       <c s="6" r="E17">
-        <v>17400</v>
+        <v>60640</v>
       </c>
       <c s="7" r="F17">
-        <v>0.0533986617691977</v>
+        <v>0.0541114957394068</v>
       </c>
       <c s="1" t="str" r="G17"/>
       <c s="1" t="str" r="H17"/>
@@ -621,22 +621,22 @@
       <c s="1" t="str" r="A18"/>
       <c s="4" t="inlineStr" r="B18">
         <is>
-          <t xml:space="preserve">GRUPOSURA</t>
+          <t xml:space="preserve">ISA</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C18">
         <is>
-          <t xml:space="preserve">GRUPO INVERSIONES SURAMERICANA</t>
+          <t xml:space="preserve">INTERCONEXION ELECTRICA S.A. E.S.P.</t>
         </is>
       </c>
       <c s="5" r="D18">
-        <v>0.0021536517955735</v>
+        <v>0.0076165367969861</v>
       </c>
       <c s="6" r="E18">
-        <v>46400</v>
+        <v>29360</v>
       </c>
       <c s="7" r="F18">
-        <v>0.0547762691384261</v>
+        <v>0.0933307959313661</v>
       </c>
       <c s="1" t="str" r="G18"/>
       <c s="1" t="str" r="H18"/>
@@ -645,22 +645,22 @@
       <c s="1" t="str" r="A19"/>
       <c s="4" t="inlineStr" r="B19">
         <is>
-          <t xml:space="preserve">ISA</t>
+          <t xml:space="preserve">MINEROS</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C19">
         <is>
-          <t xml:space="preserve">INTERCONEXION ELECTRICA S.A. E.S.P.</t>
+          <t xml:space="preserve">MINEROS S.A.</t>
         </is>
       </c>
       <c s="5" r="D19">
-        <v>0.0076417618931885</v>
+        <v>0.0015457749252731</v>
       </c>
       <c s="6" r="E19">
-        <v>22900</v>
+        <v>18720</v>
       </c>
       <c s="7" r="F19">
-        <v>0.095924151110561</v>
+        <v>0.0120771226335084</v>
       </c>
       <c s="1" t="str" r="G19"/>
       <c s="1" t="str" r="H19"/>
@@ -669,22 +669,22 @@
       <c s="1" t="str" r="A20"/>
       <c s="4" t="inlineStr" r="B20">
         <is>
-          <t xml:space="preserve">MINEROS</t>
+          <t xml:space="preserve">PEI</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C20">
         <is>
-          <t xml:space="preserve">MINEROS S.A.</t>
+          <t xml:space="preserve">PATRIMONIO AUTONOMO DE ESTRATEGIAS INMOBILIARIAS</t>
         </is>
       </c>
       <c s="5" r="D20">
-        <v>0.0015508943545145</v>
+        <v>0.0004820584601553</v>
       </c>
       <c s="6" r="E20">
-        <v>7800</v>
+        <v>73120</v>
       </c>
       <c s="7" r="F20">
-        <v>0.0066309506913336</v>
+        <v>0.0147111717424216</v>
       </c>
       <c s="1" t="str" r="G20"/>
       <c s="1" t="str" r="H20"/>
@@ -693,22 +693,22 @@
       <c s="1" t="str" r="A21"/>
       <c s="4" t="inlineStr" r="B21">
         <is>
-          <t xml:space="preserve">PEI</t>
+          <t xml:space="preserve">PFAVAL</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C21">
         <is>
-          <t xml:space="preserve">PATRIMONIO AUTONOMO DE ESTRATEGIAS INMOBILIARIAS</t>
+          <t xml:space="preserve">GRUPO AVAL ACCIONES Y VALORES S.A.</t>
         </is>
       </c>
       <c s="5" r="D21">
-        <v>0.0004836549824799</v>
+        <v>0.0714985328173631</v>
       </c>
       <c s="6" r="E21">
-        <v>69800</v>
+        <v>815</v>
       </c>
       <c s="7" r="F21">
-        <v>0.0185050417564363</v>
+        <v>0.0243201423392018</v>
       </c>
       <c s="1" t="str" r="G21"/>
       <c s="1" t="str" r="H21"/>
@@ -717,22 +717,22 @@
       <c s="1" t="str" r="A22"/>
       <c s="4" t="inlineStr" r="B22">
         <is>
-          <t xml:space="preserve">PFAVAL</t>
+          <t xml:space="preserve">PFCIBEST</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C22">
         <is>
-          <t xml:space="preserve">GRUPO AVAL ACCIONES Y VALORES S.A.</t>
+          <t xml:space="preserve">GRUPO CIBEST SA</t>
         </is>
       </c>
       <c s="5" r="D22">
-        <v>0.0715180148569536</v>
+        <v>0.0077346244631596</v>
       </c>
       <c s="6" r="E22">
-        <v>598</v>
+        <v>73300</v>
       </c>
       <c s="7" r="F22">
-        <v>0.0234431310759396</v>
+        <v>0.236621705731446</v>
       </c>
       <c s="1" t="str" r="G22"/>
       <c s="1" t="str" r="H22"/>
@@ -741,22 +741,22 @@
       <c s="1" t="str" r="A23"/>
       <c s="4" t="inlineStr" r="B23">
         <is>
-          <t xml:space="preserve">PFCIBEST</t>
+          <t xml:space="preserve">PFCORFICOL</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C23">
         <is>
-          <t xml:space="preserve">GRUPO CIBEST SA</t>
+          <t xml:space="preserve">CORPORACION FINANCIERA COLOMBIANA S.A.</t>
         </is>
       </c>
       <c s="5" r="D23">
-        <v>0.0077978712682632</v>
+        <v>0.0002809417030771</v>
       </c>
       <c s="6" r="E23">
-        <v>48840</v>
+        <v>18820</v>
       </c>
       <c s="7" r="F23">
-        <v>0.208761638715782</v>
+        <v>0.0022067198600643</v>
       </c>
       <c s="1" t="str" r="G23"/>
       <c s="1" t="str" r="H23"/>
@@ -765,22 +765,22 @@
       <c s="1" t="str" r="A24"/>
       <c s="4" t="inlineStr" r="B24">
         <is>
-          <t xml:space="preserve">PFCORFICOL</t>
+          <t xml:space="preserve">PFDAVIGRP</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C24">
         <is>
-          <t xml:space="preserve">CORPORACION FINANCIERA COLOMBIANA S.A.</t>
+          <t xml:space="preserve">DAVIVIENDA GROUP SA</t>
         </is>
       </c>
       <c s="5" r="D24">
-        <v>0.0002818721497718</v>
+        <v>0.0017037478083277</v>
       </c>
       <c s="6" r="E24">
-        <v>16300</v>
+        <v>31000</v>
       </c>
       <c s="7" r="F24">
-        <v>0.0025184814293988</v>
+        <v>0.0220433896595426</v>
       </c>
       <c s="1" t="str" r="G24"/>
       <c s="1" t="str" r="H24"/>
@@ -789,22 +789,22 @@
       <c s="1" t="str" r="A25"/>
       <c s="4" t="inlineStr" r="B25">
         <is>
-          <t xml:space="preserve">PFDAVVNDA</t>
+          <t xml:space="preserve">PFGRUPOARG</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C25">
         <is>
-          <t xml:space="preserve">BANCO DAVIVIENDA S.A</t>
+          <t xml:space="preserve">GRUPO ARGOS S.A.</t>
         </is>
       </c>
       <c s="5" r="D25">
-        <v>0.0017093904256373</v>
+        <v>0.0047462495290940</v>
       </c>
       <c s="6" r="E25">
-        <v>24080</v>
+        <v>14360</v>
       </c>
       <c s="7" r="F25">
-        <v>0.0225629941289618</v>
+        <v>0.0284456839653381</v>
       </c>
       <c s="1" t="str" r="G25"/>
       <c s="1" t="str" r="H25"/>
@@ -813,22 +813,22 @@
       <c s="1" t="str" r="A26"/>
       <c s="4" t="inlineStr" r="B26">
         <is>
-          <t xml:space="preserve">PFGRUPOARG</t>
+          <t xml:space="preserve">PFGRUPSURA</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C26">
         <is>
-          <t xml:space="preserve">GRUPO ARGOS S.A.</t>
+          <t xml:space="preserve">GRUPO INVERSIONES SURAMERICANA</t>
         </is>
       </c>
       <c s="5" r="D26">
-        <v>0.0047656347486016</v>
+        <v>0.0026434986080165</v>
       </c>
       <c s="6" r="E26">
-        <v>11160</v>
+        <v>51700</v>
       </c>
       <c s="7" r="F26">
-        <v>0.0291530454056272</v>
+        <v>0.0570401951721633</v>
       </c>
       <c s="1" t="str" r="G26"/>
       <c s="1" t="str" r="H26"/>
@@ -837,22 +837,22 @@
       <c s="1" t="str" r="A27"/>
       <c s="4" t="inlineStr" r="B27">
         <is>
-          <t xml:space="preserve">PFGRUPSURA</t>
+          <t xml:space="preserve">PROMIGAS</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C27">
         <is>
-          <t xml:space="preserve">GRUPO INVERSIONES SURAMERICANA</t>
+          <t xml:space="preserve">PROMIGAS S.A. E.S.P.</t>
         </is>
       </c>
       <c s="5" r="D27">
-        <v>0.0026529990193005</v>
+        <v>0.0019508405659527</v>
       </c>
       <c s="6" r="E27">
-        <v>36620</v>
+        <v>6740</v>
       </c>
       <c s="7" r="F27">
-        <v>0.05325426684287</v>
+        <v>0.0054877339470709</v>
       </c>
       <c s="1" t="str" r="G27"/>
       <c s="1" t="str" r="H27"/>
@@ -861,84 +861,329 @@
       <c s="1" t="str" r="A28"/>
       <c s="4" t="inlineStr" r="B28">
         <is>
-          <t xml:space="preserve">PROMIGAS</t>
+          <t xml:space="preserve">TERPEL</t>
         </is>
       </c>
       <c s="4" t="inlineStr" r="C28">
         <is>
-          <t xml:space="preserve">PROMIGAS S.A. E.S.P.</t>
+          <t xml:space="preserve">ORGANIZACION TERPEL S.A</t>
         </is>
       </c>
       <c s="5" r="D28">
-        <v>0.0019573015261323</v>
+        <v>0.0006237492080019</v>
       </c>
       <c s="6" r="E28">
-        <v>6790</v>
+        <v>19680</v>
       </c>
       <c s="7" r="F28">
-        <v>0.0072849485629925</v>
+        <v>0.0051232609269068</v>
       </c>
       <c s="1" t="str" r="G28"/>
       <c s="1" t="str" r="H28"/>
     </row>
-    <row r="29" ht="15.1" customHeight="0">
+    <row r="29" ht="18" customHeight="1">
       <c s="1" t="str" r="A29"/>
-      <c s="4" t="inlineStr" r="B29">
-        <is>
-          <t xml:space="preserve">TERPEL</t>
-        </is>
-      </c>
-      <c s="4" t="inlineStr" r="C29">
-        <is>
-          <t xml:space="preserve">ORGANIZACION TERPEL S.A</t>
-        </is>
-      </c>
-      <c s="5" r="D29">
-        <v>0.0006258149938305</v>
-      </c>
-      <c s="6" r="E29">
-        <v>14000</v>
-      </c>
-      <c s="7" r="F29">
-        <v>0.0048025620031722</v>
-      </c>
+      <c s="8" t="inlineStr" r="B29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="1" t="str" r="C29"/>
+      <c s="1" t="str" r="D29"/>
+      <c s="1" t="str" r="E29"/>
+      <c s="1" t="str" r="F29"/>
       <c s="1" t="str" r="G29"/>
       <c s="1" t="str" r="H29"/>
     </row>
-    <row r="30" ht="0.05" customHeight="1">
-      <c s="1" t="str" r="A30"/>
-      <c s="1" t="str" r="B30"/>
-      <c s="1" t="str" r="C30"/>
-      <c s="1" t="str" r="D30"/>
-      <c s="1" t="str" r="E30"/>
-      <c s="1" t="str" r="F30"/>
-      <c s="1" t="str" r="G30"/>
-      <c s="1" t="str" r="H30"/>
-    </row>
-    <row r="31" ht="17.95" customHeight="1">
-      <c s="1" t="str" r="A31"/>
-      <c s="8" t="inlineStr" r="B31">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="1" t="str" r="C31"/>
-      <c s="1" t="str" r="D31"/>
-      <c s="1" t="str" r="E31"/>
-      <c s="1" t="str" r="F31"/>
-      <c s="1" t="str" r="G31"/>
-      <c s="1" t="str" r="H31"/>
-    </row>
-    <row r="32" ht="0.05" customHeight="1"/>
   </sheetData>
   <mergeCells>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B29:G29"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="1" footer="1"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId7"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101000B9DE74DF219394999F4407EAF939737" ma:contentTypeVersion="16" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="61f219988ef49ccb21d5de35333eff96">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="261cbb30-3a0f-4b48-ae8c-721f956beb90" xmlns:ns3="2f55542a-98f6-4fa1-96c7-fc247ffc16ef" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d8fd1eb9b00aafce4fa10120426ffbf6" ns1:_="" ns2:_="" ns3:_="">
+    <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
+    <xsd:import namespace="261cbb30-3a0f-4b48-ae8c-721f956beb90"/>
+    <xsd:import namespace="2f55542a-98f6-4fa1-96c7-fc247ffc16ef"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyProperties" minOccurs="0"/>
+                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyUIAction" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="http://schemas.microsoft.com/sharepoint/v3" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="_ip_UnifiedCompliancePolicyProperties" ma:index="22" nillable="true" ma:displayName="Propiedades de la Directiva de cumplimiento unificado" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyProperties">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_ip_UnifiedCompliancePolicyUIAction" ma:index="23" nillable="true" ma:displayName="Acción de IU de la Directiva de cumplimiento unificado" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyUIAction">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="261cbb30-3a0f-4b48-ae8c-721f956beb90" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="10" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="14" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="3b40abcd-3e59-4edb-908f-3fa5816ce1d3" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="20" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="21" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2f55542a-98f6-4fa1-96c7-fc247ffc16ef" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="17" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{cd4eb19b-fdfd-4cda-a71a-c182e4a2df97}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2f55542a-98f6-4fa1-96c7-fc247ffc16ef">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Compartido con" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Detalles de uso compartido" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="2f55542a-98f6-4fa1-96c7-fc247ffc16ef" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="261cbb30-3a0f-4b48-ae8c-721f956beb90">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7634E021-178D-4FCD-925D-1064D859EF1A}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57FAE33C-C1FE-4493-86FC-281357DAC9D0}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{023A9803-8AD0-495D-AED5-2CAA6BB57AD5}"/>
 </file>
</xml_diff>